<commit_message>
katalog guncelleme - badem ezmesi + kurabi biskuvi
</commit_message>
<xml_diff>
--- a/panel/sevkiyat_sablon.xlsx
+++ b/panel/sevkiyat_sablon.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A98DEAC-AF95-401D-9B8F-2E8F08479CC2}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{2A98DEAC-AF95-401D-9B8F-2E8F08479CC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08FEB819-6BB3-4BCC-AF7C-F22519491BBA}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3696" yWindow="516" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HAMMADDE TALEP FORMU" sheetId="4" r:id="rId1"/>
@@ -19,6 +19,20 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -1565,132 +1579,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1700,9 +1588,6 @@
     </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" textRotation="90" wrapText="1"/>
@@ -1711,6 +1596,135 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2124,29 +2138,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="66"/>
-      <c r="B1" s="67"/>
-      <c r="C1" s="93" t="s">
+      <c r="A1" s="91"/>
+      <c r="B1" s="92"/>
+      <c r="C1" s="83" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="95"/>
-      <c r="I1" s="96" t="s">
+      <c r="D1" s="84"/>
+      <c r="E1" s="84"/>
+      <c r="F1" s="84"/>
+      <c r="G1" s="84"/>
+      <c r="H1" s="85"/>
+      <c r="I1" s="86" t="s">
         <v>257</v>
       </c>
-      <c r="J1" s="97"/>
+      <c r="J1" s="87"/>
       <c r="K1" s="59" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="96" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="72"/>
+      <c r="B2" s="97"/>
       <c r="C2" s="23" t="s">
         <v>18</v>
       </c>
@@ -2156,11 +2170,11 @@
       <c r="E2" s="58" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="76"/>
-      <c r="G2" s="68" t="s">
+      <c r="F2" s="98"/>
+      <c r="G2" s="93" t="s">
         <v>58</v>
       </c>
-      <c r="H2" s="69"/>
+      <c r="H2" s="94"/>
       <c r="I2" s="23" t="s">
         <v>18</v>
       </c>
@@ -2172,7 +2186,7 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="88" t="s">
         <v>57</v>
       </c>
       <c r="B3" s="33" t="s">
@@ -2185,8 +2199,8 @@
         <v>17</v>
       </c>
       <c r="E3" s="28"/>
-      <c r="F3" s="77"/>
-      <c r="G3" s="85" t="s">
+      <c r="F3" s="99"/>
+      <c r="G3" s="77" t="s">
         <v>80</v>
       </c>
       <c r="H3" s="33" t="s">
@@ -2201,7 +2215,7 @@
       <c r="K3" s="38"/>
     </row>
     <row r="4" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="64"/>
+      <c r="A4" s="89"/>
       <c r="B4" s="34" t="s">
         <v>1</v>
       </c>
@@ -2212,8 +2226,8 @@
         <v>17</v>
       </c>
       <c r="E4" s="29"/>
-      <c r="F4" s="77"/>
-      <c r="G4" s="86"/>
+      <c r="F4" s="99"/>
+      <c r="G4" s="78"/>
       <c r="H4" s="34" t="s">
         <v>32</v>
       </c>
@@ -2226,7 +2240,7 @@
       <c r="K4" s="39"/>
     </row>
     <row r="5" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="64"/>
+      <c r="A5" s="89"/>
       <c r="B5" s="34" t="s">
         <v>2</v>
       </c>
@@ -2237,8 +2251,8 @@
         <v>17</v>
       </c>
       <c r="E5" s="29"/>
-      <c r="F5" s="77"/>
-      <c r="G5" s="86"/>
+      <c r="F5" s="99"/>
+      <c r="G5" s="78"/>
       <c r="H5" s="34" t="s">
         <v>33</v>
       </c>
@@ -2251,7 +2265,7 @@
       <c r="K5" s="39"/>
     </row>
     <row r="6" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="64"/>
+      <c r="A6" s="89"/>
       <c r="B6" s="34" t="s">
         <v>3</v>
       </c>
@@ -2262,8 +2276,8 @@
         <v>17</v>
       </c>
       <c r="E6" s="29"/>
-      <c r="F6" s="77"/>
-      <c r="G6" s="86"/>
+      <c r="F6" s="99"/>
+      <c r="G6" s="78"/>
       <c r="H6" s="34" t="s">
         <v>34</v>
       </c>
@@ -2276,7 +2290,7 @@
       <c r="K6" s="39"/>
     </row>
     <row r="7" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="64"/>
+      <c r="A7" s="89"/>
       <c r="B7" s="34" t="s">
         <v>4</v>
       </c>
@@ -2287,8 +2301,8 @@
         <v>17</v>
       </c>
       <c r="E7" s="29"/>
-      <c r="F7" s="77"/>
-      <c r="G7" s="86"/>
+      <c r="F7" s="99"/>
+      <c r="G7" s="78"/>
       <c r="H7" s="34" t="s">
         <v>35</v>
       </c>
@@ -2301,7 +2315,7 @@
       <c r="K7" s="39"/>
     </row>
     <row r="8" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="64"/>
+      <c r="A8" s="89"/>
       <c r="B8" s="34" t="s">
         <v>193</v>
       </c>
@@ -2312,8 +2326,8 @@
         <v>17</v>
       </c>
       <c r="E8" s="29"/>
-      <c r="F8" s="77"/>
-      <c r="G8" s="86"/>
+      <c r="F8" s="99"/>
+      <c r="G8" s="78"/>
       <c r="H8" s="34" t="s">
         <v>36</v>
       </c>
@@ -2326,7 +2340,7 @@
       <c r="K8" s="39"/>
     </row>
     <row r="9" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="64"/>
+      <c r="A9" s="89"/>
       <c r="B9" s="34" t="s">
         <v>194</v>
       </c>
@@ -2337,8 +2351,8 @@
         <v>17</v>
       </c>
       <c r="E9" s="29"/>
-      <c r="F9" s="77"/>
-      <c r="G9" s="86"/>
+      <c r="F9" s="99"/>
+      <c r="G9" s="78"/>
       <c r="H9" s="34" t="s">
         <v>37</v>
       </c>
@@ -2351,7 +2365,7 @@
       <c r="K9" s="39"/>
     </row>
     <row r="10" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="64"/>
+      <c r="A10" s="89"/>
       <c r="B10" s="34" t="s">
         <v>5</v>
       </c>
@@ -2362,8 +2376,8 @@
         <v>17</v>
       </c>
       <c r="E10" s="29"/>
-      <c r="F10" s="77"/>
-      <c r="G10" s="86"/>
+      <c r="F10" s="99"/>
+      <c r="G10" s="78"/>
       <c r="H10" s="34" t="s">
         <v>38</v>
       </c>
@@ -2376,7 +2390,7 @@
       <c r="K10" s="39"/>
     </row>
     <row r="11" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="64"/>
+      <c r="A11" s="89"/>
       <c r="B11" s="34" t="s">
         <v>6</v>
       </c>
@@ -2387,8 +2401,8 @@
         <v>17</v>
       </c>
       <c r="E11" s="29"/>
-      <c r="F11" s="77"/>
-      <c r="G11" s="86"/>
+      <c r="F11" s="99"/>
+      <c r="G11" s="78"/>
       <c r="H11" s="34" t="s">
         <v>170</v>
       </c>
@@ -2401,7 +2415,7 @@
       <c r="K11" s="39"/>
     </row>
     <row r="12" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="64"/>
+      <c r="A12" s="89"/>
       <c r="B12" s="34" t="s">
         <v>83</v>
       </c>
@@ -2412,8 +2426,8 @@
         <v>17</v>
       </c>
       <c r="E12" s="29"/>
-      <c r="F12" s="77"/>
-      <c r="G12" s="86"/>
+      <c r="F12" s="99"/>
+      <c r="G12" s="78"/>
       <c r="H12" s="34" t="s">
         <v>47</v>
       </c>
@@ -2426,7 +2440,7 @@
       <c r="K12" s="39"/>
     </row>
     <row r="13" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="64"/>
+      <c r="A13" s="89"/>
       <c r="B13" s="34" t="s">
         <v>7</v>
       </c>
@@ -2437,8 +2451,8 @@
         <v>17</v>
       </c>
       <c r="E13" s="29"/>
-      <c r="F13" s="77"/>
-      <c r="G13" s="86"/>
+      <c r="F13" s="99"/>
+      <c r="G13" s="78"/>
       <c r="H13" s="34" t="s">
         <v>252</v>
       </c>
@@ -2451,7 +2465,7 @@
       <c r="K13" s="39"/>
     </row>
     <row r="14" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="64"/>
+      <c r="A14" s="89"/>
       <c r="B14" s="34" t="s">
         <v>8</v>
       </c>
@@ -2462,8 +2476,8 @@
         <v>17</v>
       </c>
       <c r="E14" s="29"/>
-      <c r="F14" s="77"/>
-      <c r="G14" s="86"/>
+      <c r="F14" s="99"/>
+      <c r="G14" s="78"/>
       <c r="H14" s="34" t="s">
         <v>48</v>
       </c>
@@ -2476,7 +2490,7 @@
       <c r="K14" s="39"/>
     </row>
     <row r="15" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="64"/>
+      <c r="A15" s="89"/>
       <c r="B15" s="34" t="s">
         <v>9</v>
       </c>
@@ -2487,8 +2501,8 @@
         <v>17</v>
       </c>
       <c r="E15" s="29"/>
-      <c r="F15" s="77"/>
-      <c r="G15" s="86"/>
+      <c r="F15" s="99"/>
+      <c r="G15" s="78"/>
       <c r="H15" s="34" t="s">
         <v>49</v>
       </c>
@@ -2501,7 +2515,7 @@
       <c r="K15" s="39"/>
     </row>
     <row r="16" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="64"/>
+      <c r="A16" s="89"/>
       <c r="B16" s="34" t="s">
         <v>10</v>
       </c>
@@ -2512,8 +2526,8 @@
         <v>17</v>
       </c>
       <c r="E16" s="29"/>
-      <c r="F16" s="77"/>
-      <c r="G16" s="86"/>
+      <c r="F16" s="99"/>
+      <c r="G16" s="78"/>
       <c r="H16" s="34" t="s">
         <v>201</v>
       </c>
@@ -2526,7 +2540,7 @@
       <c r="K16" s="39"/>
     </row>
     <row r="17" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="64"/>
+      <c r="A17" s="89"/>
       <c r="B17" s="34" t="s">
         <v>11</v>
       </c>
@@ -2537,8 +2551,8 @@
         <v>17</v>
       </c>
       <c r="E17" s="29"/>
-      <c r="F17" s="77"/>
-      <c r="G17" s="86"/>
+      <c r="F17" s="99"/>
+      <c r="G17" s="78"/>
       <c r="H17" s="34" t="s">
         <v>85</v>
       </c>
@@ -2551,7 +2565,7 @@
       <c r="K17" s="39"/>
     </row>
     <row r="18" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="64"/>
+      <c r="A18" s="89"/>
       <c r="B18" s="34" t="s">
         <v>12</v>
       </c>
@@ -2562,8 +2576,8 @@
         <v>17</v>
       </c>
       <c r="E18" s="29"/>
-      <c r="F18" s="77"/>
-      <c r="G18" s="86"/>
+      <c r="F18" s="99"/>
+      <c r="G18" s="78"/>
       <c r="H18" s="34" t="s">
         <v>202</v>
       </c>
@@ -2576,7 +2590,7 @@
       <c r="K18" s="39"/>
     </row>
     <row r="19" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="64"/>
+      <c r="A19" s="89"/>
       <c r="B19" s="34" t="s">
         <v>27</v>
       </c>
@@ -2587,8 +2601,8 @@
         <v>17</v>
       </c>
       <c r="E19" s="29"/>
-      <c r="F19" s="77"/>
-      <c r="G19" s="86"/>
+      <c r="F19" s="99"/>
+      <c r="G19" s="78"/>
       <c r="H19" s="34" t="s">
         <v>243</v>
       </c>
@@ -2601,7 +2615,7 @@
       <c r="K19" s="39"/>
     </row>
     <row r="20" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="64"/>
+      <c r="A20" s="89"/>
       <c r="B20" s="34" t="s">
         <v>26</v>
       </c>
@@ -2612,8 +2626,8 @@
         <v>17</v>
       </c>
       <c r="E20" s="29"/>
-      <c r="F20" s="77"/>
-      <c r="G20" s="86"/>
+      <c r="F20" s="99"/>
+      <c r="G20" s="78"/>
       <c r="H20" s="34" t="s">
         <v>244</v>
       </c>
@@ -2626,7 +2640,7 @@
       <c r="K20" s="39"/>
     </row>
     <row r="21" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="64"/>
+      <c r="A21" s="89"/>
       <c r="B21" s="34" t="s">
         <v>62</v>
       </c>
@@ -2637,8 +2651,8 @@
         <v>17</v>
       </c>
       <c r="E21" s="29"/>
-      <c r="F21" s="77"/>
-      <c r="G21" s="86"/>
+      <c r="F21" s="99"/>
+      <c r="G21" s="78"/>
       <c r="H21" s="34" t="s">
         <v>39</v>
       </c>
@@ -2651,7 +2665,7 @@
       <c r="K21" s="39"/>
     </row>
     <row r="22" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="64"/>
+      <c r="A22" s="89"/>
       <c r="B22" s="34" t="s">
         <v>77</v>
       </c>
@@ -2662,8 +2676,8 @@
         <v>17</v>
       </c>
       <c r="E22" s="29"/>
-      <c r="F22" s="77"/>
-      <c r="G22" s="86"/>
+      <c r="F22" s="99"/>
+      <c r="G22" s="78"/>
       <c r="H22" s="34" t="s">
         <v>40</v>
       </c>
@@ -2676,7 +2690,7 @@
       <c r="K22" s="39"/>
     </row>
     <row r="23" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="64"/>
+      <c r="A23" s="89"/>
       <c r="B23" s="34" t="s">
         <v>78</v>
       </c>
@@ -2687,8 +2701,8 @@
         <v>17</v>
       </c>
       <c r="E23" s="29"/>
-      <c r="F23" s="77"/>
-      <c r="G23" s="86"/>
+      <c r="F23" s="99"/>
+      <c r="G23" s="78"/>
       <c r="H23" s="34" t="s">
         <v>41</v>
       </c>
@@ -2701,7 +2715,7 @@
       <c r="K23" s="39"/>
     </row>
     <row r="24" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="64"/>
+      <c r="A24" s="89"/>
       <c r="B24" s="34" t="s">
         <v>64</v>
       </c>
@@ -2712,8 +2726,8 @@
         <v>17</v>
       </c>
       <c r="E24" s="29"/>
-      <c r="F24" s="77"/>
-      <c r="G24" s="86"/>
+      <c r="F24" s="99"/>
+      <c r="G24" s="78"/>
       <c r="H24" s="34" t="s">
         <v>42</v>
       </c>
@@ -2726,7 +2740,7 @@
       <c r="K24" s="39"/>
     </row>
     <row r="25" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="64"/>
+      <c r="A25" s="89"/>
       <c r="B25" s="34" t="s">
         <v>63</v>
       </c>
@@ -2737,8 +2751,8 @@
         <v>17</v>
       </c>
       <c r="E25" s="29"/>
-      <c r="F25" s="77"/>
-      <c r="G25" s="86"/>
+      <c r="F25" s="99"/>
+      <c r="G25" s="78"/>
       <c r="H25" s="34" t="s">
         <v>82</v>
       </c>
@@ -2751,7 +2765,7 @@
       <c r="K25" s="39"/>
     </row>
     <row r="26" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="64"/>
+      <c r="A26" s="89"/>
       <c r="B26" s="34" t="s">
         <v>76</v>
       </c>
@@ -2762,8 +2776,8 @@
         <v>17</v>
       </c>
       <c r="E26" s="29"/>
-      <c r="F26" s="77"/>
-      <c r="G26" s="86"/>
+      <c r="F26" s="99"/>
+      <c r="G26" s="78"/>
       <c r="H26" s="34" t="s">
         <v>43</v>
       </c>
@@ -2776,7 +2790,7 @@
       <c r="K26" s="39"/>
     </row>
     <row r="27" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="64"/>
+      <c r="A27" s="89"/>
       <c r="B27" s="35" t="s">
         <v>167</v>
       </c>
@@ -2787,8 +2801,8 @@
         <v>17</v>
       </c>
       <c r="E27" s="29"/>
-      <c r="F27" s="77"/>
-      <c r="G27" s="86"/>
+      <c r="F27" s="99"/>
+      <c r="G27" s="78"/>
       <c r="H27" s="34" t="s">
         <v>44</v>
       </c>
@@ -2801,7 +2815,7 @@
       <c r="K27" s="39"/>
     </row>
     <row r="28" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="64"/>
+      <c r="A28" s="89"/>
       <c r="B28" s="34" t="s">
         <v>195</v>
       </c>
@@ -2812,8 +2826,8 @@
         <v>88</v>
       </c>
       <c r="E28" s="29"/>
-      <c r="F28" s="77"/>
-      <c r="G28" s="86"/>
+      <c r="F28" s="99"/>
+      <c r="G28" s="78"/>
       <c r="H28" s="34" t="s">
         <v>245</v>
       </c>
@@ -2826,7 +2840,7 @@
       <c r="K28" s="39"/>
     </row>
     <row r="29" spans="1:11" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="65"/>
+      <c r="A29" s="90"/>
       <c r="B29" s="36" t="s">
         <v>196</v>
       </c>
@@ -2837,8 +2851,8 @@
         <v>88</v>
       </c>
       <c r="E29" s="32"/>
-      <c r="F29" s="77"/>
-      <c r="G29" s="86"/>
+      <c r="F29" s="99"/>
+      <c r="G29" s="78"/>
       <c r="H29" s="34" t="s">
         <v>45</v>
       </c>
@@ -2851,13 +2865,13 @@
       <c r="K29" s="39"/>
     </row>
     <row r="30" spans="1:11" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="70"/>
-      <c r="B30" s="70"/>
-      <c r="C30" s="70"/>
-      <c r="D30" s="70"/>
-      <c r="E30" s="70"/>
-      <c r="F30" s="77"/>
-      <c r="G30" s="86"/>
+      <c r="A30" s="95"/>
+      <c r="B30" s="95"/>
+      <c r="C30" s="95"/>
+      <c r="D30" s="95"/>
+      <c r="E30" s="95"/>
+      <c r="F30" s="99"/>
+      <c r="G30" s="78"/>
       <c r="H30" s="34" t="s">
         <v>20</v>
       </c>
@@ -2870,7 +2884,7 @@
       <c r="K30" s="39"/>
     </row>
     <row r="31" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="85" t="s">
+      <c r="A31" s="77" t="s">
         <v>75</v>
       </c>
       <c r="B31" s="33" t="s">
@@ -2883,8 +2897,8 @@
         <v>16</v>
       </c>
       <c r="E31" s="28"/>
-      <c r="F31" s="77"/>
-      <c r="G31" s="86"/>
+      <c r="F31" s="99"/>
+      <c r="G31" s="78"/>
       <c r="H31" s="34" t="s">
         <v>46</v>
       </c>
@@ -2897,7 +2911,7 @@
       <c r="K31" s="39"/>
     </row>
     <row r="32" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="86"/>
+      <c r="A32" s="78"/>
       <c r="B32" s="34" t="s">
         <v>22</v>
       </c>
@@ -2908,8 +2922,8 @@
         <v>16</v>
       </c>
       <c r="E32" s="29"/>
-      <c r="F32" s="77"/>
-      <c r="G32" s="86"/>
+      <c r="F32" s="99"/>
+      <c r="G32" s="78"/>
       <c r="H32" s="34" t="s">
         <v>209</v>
       </c>
@@ -2922,7 +2936,7 @@
       <c r="K32" s="39"/>
     </row>
     <row r="33" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="86"/>
+      <c r="A33" s="78"/>
       <c r="B33" s="34" t="s">
         <v>50</v>
       </c>
@@ -2933,8 +2947,8 @@
         <v>16</v>
       </c>
       <c r="E33" s="29"/>
-      <c r="F33" s="77"/>
-      <c r="G33" s="86"/>
+      <c r="F33" s="99"/>
+      <c r="G33" s="78"/>
       <c r="H33" s="34" t="s">
         <v>86</v>
       </c>
@@ -2947,7 +2961,7 @@
       <c r="K33" s="51"/>
     </row>
     <row r="34" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="86"/>
+      <c r="A34" s="78"/>
       <c r="B34" s="34" t="s">
         <v>51</v>
       </c>
@@ -2958,8 +2972,8 @@
         <v>16</v>
       </c>
       <c r="E34" s="29"/>
-      <c r="F34" s="77"/>
-      <c r="G34" s="86"/>
+      <c r="F34" s="99"/>
+      <c r="G34" s="78"/>
       <c r="H34" s="34" t="s">
         <v>240</v>
       </c>
@@ -2972,7 +2986,7 @@
       <c r="K34" s="39"/>
     </row>
     <row r="35" spans="1:13" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="86"/>
+      <c r="A35" s="78"/>
       <c r="B35" s="34" t="s">
         <v>208</v>
       </c>
@@ -2983,8 +2997,8 @@
         <v>16</v>
       </c>
       <c r="E35" s="29"/>
-      <c r="F35" s="77"/>
-      <c r="G35" s="87"/>
+      <c r="F35" s="99"/>
+      <c r="G35" s="79"/>
       <c r="H35" s="36" t="s">
         <v>87</v>
       </c>
@@ -2997,7 +3011,7 @@
       <c r="K35" s="43"/>
     </row>
     <row r="36" spans="1:13" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="86"/>
+      <c r="A36" s="78"/>
       <c r="B36" s="34" t="s">
         <v>30</v>
       </c>
@@ -3008,15 +3022,15 @@
         <v>17</v>
       </c>
       <c r="E36" s="29"/>
-      <c r="F36" s="77"/>
-      <c r="G36" s="73"/>
-      <c r="H36" s="74"/>
-      <c r="I36" s="74"/>
-      <c r="J36" s="74"/>
-      <c r="K36" s="75"/>
+      <c r="F36" s="99"/>
+      <c r="G36" s="72"/>
+      <c r="H36" s="73"/>
+      <c r="I36" s="73"/>
+      <c r="J36" s="73"/>
+      <c r="K36" s="74"/>
     </row>
     <row r="37" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="86"/>
+      <c r="A37" s="78"/>
       <c r="B37" s="34" t="s">
         <v>54</v>
       </c>
@@ -3027,8 +3041,8 @@
         <v>14</v>
       </c>
       <c r="E37" s="29"/>
-      <c r="F37" s="77"/>
-      <c r="G37" s="85" t="s">
+      <c r="F37" s="99"/>
+      <c r="G37" s="77" t="s">
         <v>74</v>
       </c>
       <c r="H37" s="33" t="s">
@@ -3043,19 +3057,19 @@
       <c r="K37" s="38"/>
     </row>
     <row r="38" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="86"/>
+      <c r="A38" s="78"/>
       <c r="B38" s="34" t="s">
         <v>239</v>
       </c>
       <c r="C38" s="20">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D38" s="20" t="s">
         <v>14</v>
       </c>
       <c r="E38" s="29"/>
-      <c r="F38" s="77"/>
-      <c r="G38" s="86"/>
+      <c r="F38" s="99"/>
+      <c r="G38" s="78"/>
       <c r="H38" s="34" t="s">
         <v>200</v>
       </c>
@@ -3068,19 +3082,19 @@
       <c r="K38" s="39"/>
     </row>
     <row r="39" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="86"/>
+      <c r="A39" s="78"/>
       <c r="B39" s="34" t="s">
         <v>65</v>
       </c>
       <c r="C39" s="20">
-        <v>198</v>
+        <v>12</v>
       </c>
       <c r="D39" s="20" t="s">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="E39" s="37"/>
-      <c r="F39" s="77"/>
-      <c r="G39" s="86"/>
+      <c r="F39" s="99"/>
+      <c r="G39" s="78"/>
       <c r="H39" s="34" t="s">
         <v>69</v>
       </c>
@@ -3093,7 +3107,7 @@
       <c r="K39" s="40"/>
     </row>
     <row r="40" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="86"/>
+      <c r="A40" s="78"/>
       <c r="B40" s="34" t="s">
         <v>205</v>
       </c>
@@ -3104,8 +3118,8 @@
         <v>17</v>
       </c>
       <c r="E40" s="37"/>
-      <c r="F40" s="77"/>
-      <c r="G40" s="86"/>
+      <c r="F40" s="99"/>
+      <c r="G40" s="78"/>
       <c r="H40" s="34" t="s">
         <v>197</v>
       </c>
@@ -3118,7 +3132,7 @@
       <c r="K40" s="39"/>
     </row>
     <row r="41" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="86"/>
+      <c r="A41" s="78"/>
       <c r="B41" s="34" t="s">
         <v>203</v>
       </c>
@@ -3129,8 +3143,8 @@
         <v>17</v>
       </c>
       <c r="E41" s="37"/>
-      <c r="F41" s="77"/>
-      <c r="G41" s="86"/>
+      <c r="F41" s="99"/>
+      <c r="G41" s="78"/>
       <c r="H41" s="34" t="s">
         <v>231</v>
       </c>
@@ -3143,7 +3157,7 @@
       <c r="K41" s="39"/>
     </row>
     <row r="42" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="86"/>
+      <c r="A42" s="78"/>
       <c r="B42" s="34" t="s">
         <v>204</v>
       </c>
@@ -3154,8 +3168,8 @@
         <v>17</v>
       </c>
       <c r="E42" s="37"/>
-      <c r="F42" s="77"/>
-      <c r="G42" s="86"/>
+      <c r="F42" s="99"/>
+      <c r="G42" s="78"/>
       <c r="H42" s="34" t="s">
         <v>171</v>
       </c>
@@ -3169,7 +3183,7 @@
       <c r="M42" s="46"/>
     </row>
     <row r="43" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="86"/>
+      <c r="A43" s="78"/>
       <c r="B43" s="34" t="s">
         <v>222</v>
       </c>
@@ -3180,8 +3194,8 @@
         <v>14</v>
       </c>
       <c r="E43" s="37"/>
-      <c r="F43" s="77"/>
-      <c r="G43" s="86"/>
+      <c r="F43" s="99"/>
+      <c r="G43" s="78"/>
       <c r="H43" s="34" t="s">
         <v>172</v>
       </c>
@@ -3195,7 +3209,7 @@
       <c r="M43" s="46"/>
     </row>
     <row r="44" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="86"/>
+      <c r="A44" s="78"/>
       <c r="B44" s="34" t="s">
         <v>211</v>
       </c>
@@ -3206,8 +3220,8 @@
         <v>14</v>
       </c>
       <c r="E44" s="37"/>
-      <c r="F44" s="77"/>
-      <c r="G44" s="86"/>
+      <c r="F44" s="99"/>
+      <c r="G44" s="78"/>
       <c r="H44" s="34" t="s">
         <v>71</v>
       </c>
@@ -3221,7 +3235,7 @@
       <c r="M44" s="46"/>
     </row>
     <row r="45" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="86"/>
+      <c r="A45" s="78"/>
       <c r="B45" s="34" t="s">
         <v>264</v>
       </c>
@@ -3232,8 +3246,8 @@
         <v>68</v>
       </c>
       <c r="E45" s="37"/>
-      <c r="F45" s="77"/>
-      <c r="G45" s="86"/>
+      <c r="F45" s="99"/>
+      <c r="G45" s="78"/>
       <c r="H45" s="34" t="s">
         <v>198</v>
       </c>
@@ -3247,7 +3261,7 @@
       <c r="M45" s="46"/>
     </row>
     <row r="46" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="86"/>
+      <c r="A46" s="78"/>
       <c r="B46" s="34" t="s">
         <v>265</v>
       </c>
@@ -3258,8 +3272,8 @@
         <v>68</v>
       </c>
       <c r="E46" s="37"/>
-      <c r="F46" s="77"/>
-      <c r="G46" s="86"/>
+      <c r="F46" s="99"/>
+      <c r="G46" s="78"/>
       <c r="H46" s="34" t="s">
         <v>70</v>
       </c>
@@ -3273,7 +3287,7 @@
       <c r="M46" s="46"/>
     </row>
     <row r="47" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="86"/>
+      <c r="A47" s="78"/>
       <c r="B47" s="34" t="s">
         <v>266</v>
       </c>
@@ -3284,8 +3298,8 @@
         <v>68</v>
       </c>
       <c r="E47" s="37"/>
-      <c r="F47" s="77"/>
-      <c r="G47" s="86"/>
+      <c r="F47" s="99"/>
+      <c r="G47" s="78"/>
       <c r="H47" s="34" t="s">
         <v>199</v>
       </c>
@@ -3299,7 +3313,7 @@
       <c r="M47" s="46"/>
     </row>
     <row r="48" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="86"/>
+      <c r="A48" s="78"/>
       <c r="B48" s="34" t="s">
         <v>66</v>
       </c>
@@ -3310,8 +3324,8 @@
         <v>68</v>
       </c>
       <c r="E48" s="37"/>
-      <c r="F48" s="77"/>
-      <c r="G48" s="86"/>
+      <c r="F48" s="99"/>
+      <c r="G48" s="78"/>
       <c r="H48" s="34" t="s">
         <v>250</v>
       </c>
@@ -3325,7 +3339,7 @@
       <c r="M48" s="46"/>
     </row>
     <row r="49" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="86"/>
+      <c r="A49" s="78"/>
       <c r="B49" s="34" t="s">
         <v>249</v>
       </c>
@@ -3336,8 +3350,8 @@
         <v>68</v>
       </c>
       <c r="E49" s="37"/>
-      <c r="F49" s="77"/>
-      <c r="G49" s="86"/>
+      <c r="F49" s="99"/>
+      <c r="G49" s="78"/>
       <c r="H49" s="34" t="s">
         <v>251</v>
       </c>
@@ -3351,7 +3365,7 @@
       <c r="M49" s="46"/>
     </row>
     <row r="50" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="86"/>
+      <c r="A50" s="78"/>
       <c r="B50" s="34" t="s">
         <v>236</v>
       </c>
@@ -3362,8 +3376,8 @@
         <v>17</v>
       </c>
       <c r="E50" s="37"/>
-      <c r="F50" s="77"/>
-      <c r="G50" s="86"/>
+      <c r="F50" s="99"/>
+      <c r="G50" s="78"/>
       <c r="H50" s="34" t="s">
         <v>232</v>
       </c>
@@ -3377,7 +3391,7 @@
       <c r="M50" s="46"/>
     </row>
     <row r="51" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="86"/>
+      <c r="A51" s="78"/>
       <c r="B51" s="34" t="s">
         <v>237</v>
       </c>
@@ -3388,8 +3402,8 @@
         <v>238</v>
       </c>
       <c r="E51" s="37"/>
-      <c r="F51" s="77"/>
-      <c r="G51" s="86"/>
+      <c r="F51" s="99"/>
+      <c r="G51" s="78"/>
       <c r="H51" s="34" t="s">
         <v>233</v>
       </c>
@@ -3403,7 +3417,7 @@
       <c r="M51" s="46"/>
     </row>
     <row r="52" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="86"/>
+      <c r="A52" s="78"/>
       <c r="B52" s="34" t="s">
         <v>241</v>
       </c>
@@ -3414,8 +3428,8 @@
         <v>68</v>
       </c>
       <c r="E52" s="37"/>
-      <c r="F52" s="77"/>
-      <c r="G52" s="86"/>
+      <c r="F52" s="99"/>
+      <c r="G52" s="78"/>
       <c r="H52" s="34" t="s">
         <v>234</v>
       </c>
@@ -3429,7 +3443,7 @@
       <c r="M52" s="46"/>
     </row>
     <row r="53" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="86"/>
+      <c r="A53" s="78"/>
       <c r="B53" s="34" t="s">
         <v>242</v>
       </c>
@@ -3440,22 +3454,22 @@
         <v>68</v>
       </c>
       <c r="E53" s="37"/>
-      <c r="F53" s="77"/>
-      <c r="G53" s="86"/>
-      <c r="H53" s="105" t="s">
+      <c r="F53" s="99"/>
+      <c r="G53" s="78"/>
+      <c r="H53" s="63" t="s">
         <v>235</v>
       </c>
-      <c r="I53" s="108">
-        <v>1</v>
-      </c>
-      <c r="J53" s="106" t="s">
+      <c r="I53" s="66">
+        <v>1</v>
+      </c>
+      <c r="J53" s="64" t="s">
         <v>17</v>
       </c>
       <c r="K53" s="47"/>
       <c r="M53" s="46"/>
     </row>
     <row r="54" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="86"/>
+      <c r="A54" s="78"/>
       <c r="B54" s="34" t="s">
         <v>248</v>
       </c>
@@ -3466,48 +3480,48 @@
         <v>68</v>
       </c>
       <c r="E54" s="37"/>
-      <c r="F54" s="77"/>
-      <c r="G54" s="86"/>
-      <c r="H54" s="105" t="s">
+      <c r="F54" s="99"/>
+      <c r="G54" s="78"/>
+      <c r="H54" s="63" t="s">
         <v>267</v>
       </c>
-      <c r="I54" s="108">
-        <v>1</v>
-      </c>
-      <c r="J54" s="106" t="s">
+      <c r="I54" s="66">
+        <v>1</v>
+      </c>
+      <c r="J54" s="64" t="s">
         <v>17</v>
       </c>
       <c r="K54" s="47"/>
       <c r="M54" s="46"/>
     </row>
     <row r="55" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="86"/>
-      <c r="B55" s="105" t="s">
+      <c r="A55" s="78"/>
+      <c r="B55" s="63" t="s">
         <v>254</v>
       </c>
-      <c r="C55" s="106">
+      <c r="C55" s="64">
         <v>1000</v>
       </c>
-      <c r="D55" s="106" t="s">
+      <c r="D55" s="64" t="s">
         <v>68</v>
       </c>
-      <c r="E55" s="107"/>
-      <c r="F55" s="77"/>
-      <c r="G55" s="86"/>
-      <c r="H55" s="105" t="s">
+      <c r="E55" s="65"/>
+      <c r="F55" s="99"/>
+      <c r="G55" s="78"/>
+      <c r="H55" s="63" t="s">
         <v>262</v>
       </c>
-      <c r="I55" s="108">
-        <v>1</v>
-      </c>
-      <c r="J55" s="106" t="s">
+      <c r="I55" s="66">
+        <v>1</v>
+      </c>
+      <c r="J55" s="64" t="s">
         <v>17</v>
       </c>
       <c r="K55" s="47"/>
       <c r="M55" s="46"/>
     </row>
     <row r="56" spans="1:19" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="87"/>
+      <c r="A56" s="79"/>
       <c r="B56" s="36" t="s">
         <v>261</v>
       </c>
@@ -3518,8 +3532,8 @@
         <v>68</v>
       </c>
       <c r="E56" s="52"/>
-      <c r="F56" s="77"/>
-      <c r="G56" s="87"/>
+      <c r="F56" s="99"/>
+      <c r="G56" s="79"/>
       <c r="H56" s="36" t="s">
         <v>263</v>
       </c>
@@ -3532,21 +3546,21 @@
       <c r="K56" s="47"/>
     </row>
     <row r="57" spans="1:19" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="73"/>
-      <c r="B57" s="74"/>
-      <c r="C57" s="74"/>
-      <c r="D57" s="74"/>
-      <c r="E57" s="75"/>
-      <c r="F57" s="77"/>
-      <c r="G57" s="90"/>
-      <c r="H57" s="91"/>
-      <c r="I57" s="91"/>
-      <c r="J57" s="91"/>
-      <c r="K57" s="92"/>
+      <c r="A57" s="72"/>
+      <c r="B57" s="73"/>
+      <c r="C57" s="73"/>
+      <c r="D57" s="73"/>
+      <c r="E57" s="74"/>
+      <c r="F57" s="99"/>
+      <c r="G57" s="80"/>
+      <c r="H57" s="81"/>
+      <c r="I57" s="81"/>
+      <c r="J57" s="81"/>
+      <c r="K57" s="82"/>
       <c r="S57" s="46"/>
     </row>
     <row r="58" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="63" t="s">
+      <c r="A58" s="88" t="s">
         <v>212</v>
       </c>
       <c r="B58" s="33" t="s">
@@ -3559,8 +3573,8 @@
         <v>14</v>
       </c>
       <c r="E58" s="53"/>
-      <c r="F58" s="77"/>
-      <c r="G58" s="79" t="s">
+      <c r="F58" s="99"/>
+      <c r="G58" s="101" t="s">
         <v>218</v>
       </c>
       <c r="H58" s="33" t="s">
@@ -3576,7 +3590,7 @@
       <c r="S58" s="46"/>
     </row>
     <row r="59" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="64"/>
+      <c r="A59" s="89"/>
       <c r="B59" s="34" t="s">
         <v>29</v>
       </c>
@@ -3587,8 +3601,8 @@
         <v>14</v>
       </c>
       <c r="E59" s="54"/>
-      <c r="F59" s="77"/>
-      <c r="G59" s="80"/>
+      <c r="F59" s="99"/>
+      <c r="G59" s="102"/>
       <c r="H59" s="34" t="s">
         <v>220</v>
       </c>
@@ -3603,7 +3617,7 @@
       <c r="S59" s="46"/>
     </row>
     <row r="60" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="64"/>
+      <c r="A60" s="89"/>
       <c r="B60" s="34" t="s">
         <v>23</v>
       </c>
@@ -3614,8 +3628,8 @@
         <v>14</v>
       </c>
       <c r="E60" s="54"/>
-      <c r="F60" s="77"/>
-      <c r="G60" s="80"/>
+      <c r="F60" s="99"/>
+      <c r="G60" s="102"/>
       <c r="H60" s="34" t="s">
         <v>230</v>
       </c>
@@ -3630,7 +3644,7 @@
       <c r="S60" s="46"/>
     </row>
     <row r="61" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="64"/>
+      <c r="A61" s="89"/>
       <c r="B61" s="34" t="s">
         <v>207</v>
       </c>
@@ -3641,8 +3655,8 @@
         <v>17</v>
       </c>
       <c r="E61" s="54"/>
-      <c r="F61" s="77"/>
-      <c r="G61" s="80"/>
+      <c r="F61" s="99"/>
+      <c r="G61" s="102"/>
       <c r="H61" s="34" t="s">
         <v>221</v>
       </c>
@@ -3657,7 +3671,7 @@
       <c r="S61" s="46"/>
     </row>
     <row r="62" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="64"/>
+      <c r="A62" s="89"/>
       <c r="B62" s="34" t="s">
         <v>168</v>
       </c>
@@ -3668,8 +3682,8 @@
         <v>17</v>
       </c>
       <c r="E62" s="54"/>
-      <c r="F62" s="77"/>
-      <c r="G62" s="80"/>
+      <c r="F62" s="99"/>
+      <c r="G62" s="102"/>
       <c r="H62" s="34" t="s">
         <v>255</v>
       </c>
@@ -3683,7 +3697,7 @@
       <c r="O62" s="46"/>
     </row>
     <row r="63" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="64"/>
+      <c r="A63" s="89"/>
       <c r="B63" s="34" t="s">
         <v>217</v>
       </c>
@@ -3694,22 +3708,22 @@
         <v>149</v>
       </c>
       <c r="E63" s="54"/>
-      <c r="F63" s="77"/>
-      <c r="G63" s="109"/>
-      <c r="H63" s="105" t="s">
+      <c r="F63" s="99"/>
+      <c r="G63" s="103"/>
+      <c r="H63" s="63" t="s">
         <v>268</v>
       </c>
-      <c r="I63" s="106">
-        <v>1</v>
-      </c>
-      <c r="J63" s="106" t="s">
-        <v>17</v>
-      </c>
-      <c r="K63" s="110"/>
+      <c r="I63" s="64">
+        <v>1</v>
+      </c>
+      <c r="J63" s="64" t="s">
+        <v>17</v>
+      </c>
+      <c r="K63" s="67"/>
       <c r="M63" s="17"/>
     </row>
     <row r="64" spans="1:19" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="64"/>
+      <c r="A64" s="89"/>
       <c r="B64" s="34" t="s">
         <v>216</v>
       </c>
@@ -3719,9 +3733,12 @@
       <c r="D64" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="E64" s="54"/>
-      <c r="F64" s="77"/>
-      <c r="G64" s="81"/>
+      <c r="E64" s="54">
+        <f>-C39</f>
+        <v>-12</v>
+      </c>
+      <c r="F64" s="99"/>
+      <c r="G64" s="104"/>
       <c r="H64" s="36" t="s">
         <v>256</v>
       </c>
@@ -3735,7 +3752,7 @@
       <c r="M64" s="17"/>
     </row>
     <row r="65" spans="1:11" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="64"/>
+      <c r="A65" s="89"/>
       <c r="B65" s="34" t="s">
         <v>215</v>
       </c>
@@ -3746,15 +3763,15 @@
         <v>149</v>
       </c>
       <c r="E65" s="54"/>
-      <c r="F65" s="77"/>
-      <c r="G65" s="82"/>
-      <c r="H65" s="83"/>
-      <c r="I65" s="83"/>
-      <c r="J65" s="83"/>
-      <c r="K65" s="84"/>
+      <c r="F65" s="99"/>
+      <c r="G65" s="105"/>
+      <c r="H65" s="106"/>
+      <c r="I65" s="106"/>
+      <c r="J65" s="106"/>
+      <c r="K65" s="107"/>
     </row>
     <row r="66" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="64"/>
+      <c r="A66" s="89"/>
       <c r="B66" s="34" t="s">
         <v>214</v>
       </c>
@@ -3765,8 +3782,8 @@
         <v>149</v>
       </c>
       <c r="E66" s="54"/>
-      <c r="F66" s="77"/>
-      <c r="G66" s="88" t="s">
+      <c r="F66" s="99"/>
+      <c r="G66" s="75" t="s">
         <v>229</v>
       </c>
       <c r="H66" s="25" t="s">
@@ -3781,7 +3798,7 @@
       <c r="K66" s="44"/>
     </row>
     <row r="67" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="64"/>
+      <c r="A67" s="89"/>
       <c r="B67" s="34" t="s">
         <v>213</v>
       </c>
@@ -3792,8 +3809,8 @@
         <v>149</v>
       </c>
       <c r="E67" s="54"/>
-      <c r="F67" s="77"/>
-      <c r="G67" s="89"/>
+      <c r="F67" s="99"/>
+      <c r="G67" s="76"/>
       <c r="H67" s="18" t="s">
         <v>225</v>
       </c>
@@ -3806,7 +3823,7 @@
       <c r="K67" s="39"/>
     </row>
     <row r="68" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="64"/>
+      <c r="A68" s="89"/>
       <c r="B68" s="34" t="s">
         <v>223</v>
       </c>
@@ -3817,8 +3834,8 @@
         <v>149</v>
       </c>
       <c r="E68" s="54"/>
-      <c r="F68" s="77"/>
-      <c r="G68" s="89"/>
+      <c r="F68" s="99"/>
+      <c r="G68" s="76"/>
       <c r="H68" s="18" t="s">
         <v>247</v>
       </c>
@@ -3831,7 +3848,7 @@
       <c r="K68" s="39"/>
     </row>
     <row r="69" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="64"/>
+      <c r="A69" s="89"/>
       <c r="B69" s="34" t="s">
         <v>24</v>
       </c>
@@ -3842,8 +3859,8 @@
         <v>17</v>
       </c>
       <c r="E69" s="54"/>
-      <c r="F69" s="77"/>
-      <c r="G69" s="89"/>
+      <c r="F69" s="99"/>
+      <c r="G69" s="76"/>
       <c r="H69" s="18" t="s">
         <v>226</v>
       </c>
@@ -3856,7 +3873,7 @@
       <c r="K69" s="39"/>
     </row>
     <row r="70" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="64"/>
+      <c r="A70" s="89"/>
       <c r="B70" s="34" t="s">
         <v>55</v>
       </c>
@@ -3867,8 +3884,8 @@
         <v>17</v>
       </c>
       <c r="E70" s="54"/>
-      <c r="F70" s="77"/>
-      <c r="G70" s="89"/>
+      <c r="F70" s="99"/>
+      <c r="G70" s="76"/>
       <c r="H70" s="18" t="s">
         <v>227</v>
       </c>
@@ -3881,7 +3898,7 @@
       <c r="K70" s="39"/>
     </row>
     <row r="71" spans="1:11" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="64"/>
+      <c r="A71" s="89"/>
       <c r="B71" s="34" t="s">
         <v>56</v>
       </c>
@@ -3892,8 +3909,8 @@
         <v>17</v>
       </c>
       <c r="E71" s="54"/>
-      <c r="F71" s="77"/>
-      <c r="G71" s="89"/>
+      <c r="F71" s="99"/>
+      <c r="G71" s="76"/>
       <c r="H71" s="18" t="s">
         <v>228</v>
       </c>
@@ -3906,13 +3923,13 @@
       <c r="K71" s="39"/>
     </row>
     <row r="72" spans="1:11" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="73"/>
-      <c r="B72" s="74"/>
-      <c r="C72" s="74"/>
-      <c r="D72" s="74"/>
-      <c r="E72" s="75"/>
-      <c r="F72" s="77"/>
-      <c r="G72" s="89"/>
+      <c r="A72" s="72"/>
+      <c r="B72" s="73"/>
+      <c r="C72" s="73"/>
+      <c r="D72" s="73"/>
+      <c r="E72" s="74"/>
+      <c r="F72" s="99"/>
+      <c r="G72" s="76"/>
       <c r="H72" s="18" t="s">
         <v>253</v>
       </c>
@@ -3925,7 +3942,7 @@
       <c r="K72" s="39"/>
     </row>
     <row r="73" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="63" t="s">
+      <c r="A73" s="88" t="s">
         <v>81</v>
       </c>
       <c r="B73" s="33" t="s">
@@ -3938,8 +3955,8 @@
         <v>17</v>
       </c>
       <c r="E73" s="53"/>
-      <c r="F73" s="77"/>
-      <c r="G73" s="89"/>
+      <c r="F73" s="99"/>
+      <c r="G73" s="76"/>
       <c r="H73" s="18" t="s">
         <v>259</v>
       </c>
@@ -3952,7 +3969,7 @@
       <c r="K73" s="39"/>
     </row>
     <row r="74" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="64"/>
+      <c r="A74" s="89"/>
       <c r="B74" s="34" t="s">
         <v>53</v>
       </c>
@@ -3963,8 +3980,8 @@
         <v>17</v>
       </c>
       <c r="E74" s="54"/>
-      <c r="F74" s="77"/>
-      <c r="G74" s="89"/>
+      <c r="F74" s="99"/>
+      <c r="G74" s="76"/>
       <c r="H74" s="18" t="s">
         <v>269</v>
       </c>
@@ -3977,7 +3994,7 @@
       <c r="K74" s="39"/>
     </row>
     <row r="75" spans="1:11" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="64"/>
+      <c r="A75" s="89"/>
       <c r="B75" s="34" t="s">
         <v>25</v>
       </c>
@@ -3988,8 +4005,8 @@
         <v>17</v>
       </c>
       <c r="E75" s="54"/>
-      <c r="F75" s="77"/>
-      <c r="G75" s="89"/>
+      <c r="F75" s="99"/>
+      <c r="G75" s="76"/>
       <c r="H75" s="18" t="s">
         <v>270</v>
       </c>
@@ -4002,7 +4019,7 @@
       <c r="K75" s="39"/>
     </row>
     <row r="76" spans="1:11" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="64"/>
+      <c r="A76" s="89"/>
       <c r="B76" s="34" t="s">
         <v>59</v>
       </c>
@@ -4013,15 +4030,15 @@
         <v>17</v>
       </c>
       <c r="E76" s="49"/>
-      <c r="F76" s="77"/>
-      <c r="G76" s="82"/>
-      <c r="H76" s="83"/>
-      <c r="I76" s="83"/>
-      <c r="J76" s="83"/>
-      <c r="K76" s="84"/>
+      <c r="F76" s="99"/>
+      <c r="G76" s="105"/>
+      <c r="H76" s="106"/>
+      <c r="I76" s="106"/>
+      <c r="J76" s="106"/>
+      <c r="K76" s="107"/>
     </row>
     <row r="77" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="64"/>
+      <c r="A77" s="89"/>
       <c r="B77" s="34" t="s">
         <v>60</v>
       </c>
@@ -4032,8 +4049,8 @@
         <v>17</v>
       </c>
       <c r="E77" s="29"/>
-      <c r="F77" s="77"/>
-      <c r="G77" s="63" t="s">
+      <c r="F77" s="99"/>
+      <c r="G77" s="88" t="s">
         <v>246</v>
       </c>
       <c r="H77" s="33"/>
@@ -4042,7 +4059,7 @@
       <c r="K77" s="38"/>
     </row>
     <row r="78" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="64"/>
+      <c r="A78" s="89"/>
       <c r="B78" s="34" t="s">
         <v>61</v>
       </c>
@@ -4053,15 +4070,15 @@
         <v>17</v>
       </c>
       <c r="E78" s="29"/>
-      <c r="F78" s="77"/>
-      <c r="G78" s="64"/>
+      <c r="F78" s="99"/>
+      <c r="G78" s="89"/>
       <c r="H78" s="60"/>
       <c r="I78" s="48"/>
       <c r="J78" s="48"/>
       <c r="K78" s="49"/>
     </row>
     <row r="79" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="64"/>
+      <c r="A79" s="89"/>
       <c r="B79" s="34" t="s">
         <v>72</v>
       </c>
@@ -4072,15 +4089,15 @@
         <v>17</v>
       </c>
       <c r="E79" s="29"/>
-      <c r="F79" s="77"/>
-      <c r="G79" s="64"/>
+      <c r="F79" s="99"/>
+      <c r="G79" s="89"/>
       <c r="H79" s="61"/>
       <c r="I79" s="21"/>
       <c r="J79" s="21"/>
       <c r="K79" s="55"/>
     </row>
     <row r="80" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="64"/>
+      <c r="A80" s="89"/>
       <c r="B80" s="34" t="s">
         <v>73</v>
       </c>
@@ -4091,15 +4108,15 @@
         <v>17</v>
       </c>
       <c r="E80" s="29"/>
-      <c r="F80" s="77"/>
-      <c r="G80" s="64"/>
+      <c r="F80" s="99"/>
+      <c r="G80" s="89"/>
       <c r="H80" s="34"/>
       <c r="I80" s="21"/>
       <c r="J80" s="21"/>
       <c r="K80" s="41"/>
     </row>
     <row r="81" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="64"/>
+      <c r="A81" s="89"/>
       <c r="B81" s="34" t="s">
         <v>260</v>
       </c>
@@ -4110,15 +4127,15 @@
         <v>17</v>
       </c>
       <c r="E81" s="29"/>
-      <c r="F81" s="77"/>
-      <c r="G81" s="64"/>
+      <c r="F81" s="99"/>
+      <c r="G81" s="89"/>
       <c r="H81" s="34"/>
       <c r="I81" s="22"/>
       <c r="J81" s="22"/>
       <c r="K81" s="42"/>
     </row>
     <row r="82" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="64"/>
+      <c r="A82" s="89"/>
       <c r="B82" s="34" t="s">
         <v>173</v>
       </c>
@@ -4129,15 +4146,15 @@
         <v>17</v>
       </c>
       <c r="E82" s="29"/>
-      <c r="F82" s="77"/>
-      <c r="G82" s="64"/>
+      <c r="F82" s="99"/>
+      <c r="G82" s="89"/>
       <c r="H82" s="34"/>
       <c r="I82" s="22"/>
       <c r="J82" s="22"/>
       <c r="K82" s="42"/>
     </row>
     <row r="83" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="64"/>
+      <c r="A83" s="89"/>
       <c r="B83" s="34" t="s">
         <v>174</v>
       </c>
@@ -4148,15 +4165,15 @@
         <v>17</v>
       </c>
       <c r="E83" s="29"/>
-      <c r="F83" s="77"/>
-      <c r="G83" s="64"/>
+      <c r="F83" s="99"/>
+      <c r="G83" s="89"/>
       <c r="H83" s="62"/>
       <c r="I83" s="18"/>
       <c r="J83" s="22"/>
       <c r="K83" s="42"/>
     </row>
     <row r="84" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="64"/>
+      <c r="A84" s="89"/>
       <c r="B84" s="34" t="s">
         <v>169</v>
       </c>
@@ -4167,15 +4184,15 @@
         <v>17</v>
       </c>
       <c r="E84" s="29"/>
-      <c r="F84" s="77"/>
-      <c r="G84" s="64"/>
+      <c r="F84" s="99"/>
+      <c r="G84" s="89"/>
       <c r="H84" s="62"/>
       <c r="I84" s="18"/>
       <c r="J84" s="22"/>
       <c r="K84" s="42"/>
     </row>
     <row r="85" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="64"/>
+      <c r="A85" s="89"/>
       <c r="B85" s="34" t="s">
         <v>84</v>
       </c>
@@ -4186,15 +4203,15 @@
         <v>17</v>
       </c>
       <c r="E85" s="29"/>
-      <c r="F85" s="77"/>
-      <c r="G85" s="64"/>
+      <c r="F85" s="99"/>
+      <c r="G85" s="89"/>
       <c r="H85" s="62"/>
       <c r="I85" s="18"/>
       <c r="J85" s="22"/>
       <c r="K85" s="42"/>
     </row>
     <row r="86" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A86" s="65"/>
+      <c r="A86" s="90"/>
       <c r="B86" s="36" t="s">
         <v>67</v>
       </c>
@@ -4205,24 +4222,18 @@
         <v>16</v>
       </c>
       <c r="E86" s="32"/>
-      <c r="F86" s="78"/>
-      <c r="G86" s="65"/>
-      <c r="H86" s="111"/>
-      <c r="I86" s="112"/>
-      <c r="J86" s="113"/>
-      <c r="K86" s="114"/>
+      <c r="F86" s="100"/>
+      <c r="G86" s="90"/>
+      <c r="H86" s="68"/>
+      <c r="I86" s="69"/>
+      <c r="J86" s="70"/>
+      <c r="K86" s="71"/>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.3">
       <c r="F87" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="G36:K36"/>
-    <mergeCell ref="G66:G75"/>
-    <mergeCell ref="G37:G56"/>
-    <mergeCell ref="G57:K57"/>
-    <mergeCell ref="C1:H1"/>
-    <mergeCell ref="I1:J1"/>
     <mergeCell ref="G77:G86"/>
     <mergeCell ref="A73:A86"/>
     <mergeCell ref="A1:B1"/>
@@ -4239,6 +4250,12 @@
     <mergeCell ref="A57:E57"/>
     <mergeCell ref="A58:A71"/>
     <mergeCell ref="G3:G35"/>
+    <mergeCell ref="G36:K36"/>
+    <mergeCell ref="G66:G75"/>
+    <mergeCell ref="G37:G56"/>
+    <mergeCell ref="G57:K57"/>
+    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.11811023622047245" right="0.11811023622047245" top="0.15748031496062992" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -4265,25 +4282,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="99"/>
-      <c r="B1" s="101"/>
-      <c r="C1" s="99" t="s">
+      <c r="A1" s="111"/>
+      <c r="B1" s="113"/>
+      <c r="C1" s="111" t="s">
         <v>148</v>
       </c>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
-      <c r="F1" s="100"/>
-      <c r="G1" s="101"/>
+      <c r="D1" s="112"/>
+      <c r="E1" s="112"/>
+      <c r="F1" s="112"/>
+      <c r="G1" s="113"/>
     </row>
     <row r="2" spans="1:7" ht="40.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="102" t="s">
+      <c r="B2" s="114" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="102"/>
-      <c r="D2" s="102"/>
+      <c r="C2" s="114"/>
+      <c r="D2" s="114"/>
       <c r="E2" s="11" t="s">
         <v>18</v>
       </c>
@@ -4298,11 +4315,11 @@
       <c r="A3" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="98" t="s">
+      <c r="B3" s="108" t="s">
         <v>175</v>
       </c>
-      <c r="C3" s="98"/>
-      <c r="D3" s="98"/>
+      <c r="C3" s="108"/>
+      <c r="D3" s="108"/>
       <c r="E3" s="8">
         <v>15</v>
       </c>
@@ -4315,11 +4332,11 @@
       <c r="A4" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="B4" s="98" t="s">
+      <c r="B4" s="108" t="s">
         <v>89</v>
       </c>
-      <c r="C4" s="98"/>
-      <c r="D4" s="98"/>
+      <c r="C4" s="108"/>
+      <c r="D4" s="108"/>
       <c r="E4" s="8">
         <v>20</v>
       </c>
@@ -4332,11 +4349,11 @@
       <c r="A5" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="B5" s="98" t="s">
+      <c r="B5" s="108" t="s">
         <v>150</v>
       </c>
-      <c r="C5" s="98"/>
-      <c r="D5" s="98"/>
+      <c r="C5" s="108"/>
+      <c r="D5" s="108"/>
       <c r="E5" s="8">
         <v>18</v>
       </c>
@@ -4349,11 +4366,11 @@
       <c r="A6" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="B6" s="98" t="s">
+      <c r="B6" s="108" t="s">
         <v>151</v>
       </c>
-      <c r="C6" s="98"/>
-      <c r="D6" s="98"/>
+      <c r="C6" s="108"/>
+      <c r="D6" s="108"/>
       <c r="E6" s="8">
         <v>12</v>
       </c>
@@ -4366,11 +4383,11 @@
       <c r="A7" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="B7" s="98" t="s">
+      <c r="B7" s="108" t="s">
         <v>162</v>
       </c>
-      <c r="C7" s="98"/>
-      <c r="D7" s="98"/>
+      <c r="C7" s="108"/>
+      <c r="D7" s="108"/>
       <c r="E7" s="8">
         <v>12</v>
       </c>
@@ -4383,11 +4400,11 @@
       <c r="A8" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="98" t="s">
+      <c r="B8" s="108" t="s">
         <v>161</v>
       </c>
-      <c r="C8" s="98"/>
-      <c r="D8" s="98"/>
+      <c r="C8" s="108"/>
+      <c r="D8" s="108"/>
       <c r="E8" s="15">
         <v>6</v>
       </c>
@@ -4400,11 +4417,11 @@
       <c r="A9" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="B9" s="98" t="s">
+      <c r="B9" s="108" t="s">
         <v>152</v>
       </c>
-      <c r="C9" s="98"/>
-      <c r="D9" s="98"/>
+      <c r="C9" s="108"/>
+      <c r="D9" s="108"/>
       <c r="E9" s="8">
         <v>6</v>
       </c>
@@ -4417,11 +4434,11 @@
       <c r="A10" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="B10" s="98" t="s">
+      <c r="B10" s="108" t="s">
         <v>158</v>
       </c>
-      <c r="C10" s="98"/>
-      <c r="D10" s="98"/>
+      <c r="C10" s="108"/>
+      <c r="D10" s="108"/>
       <c r="E10" s="15">
         <v>6</v>
       </c>
@@ -4434,11 +4451,11 @@
       <c r="A11" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="B11" s="98" t="s">
+      <c r="B11" s="108" t="s">
         <v>90</v>
       </c>
-      <c r="C11" s="98"/>
-      <c r="D11" s="98"/>
+      <c r="C11" s="108"/>
+      <c r="D11" s="108"/>
       <c r="E11" s="8">
         <v>1</v>
       </c>
@@ -4451,11 +4468,11 @@
       <c r="A12" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="B12" s="98" t="s">
+      <c r="B12" s="108" t="s">
         <v>91</v>
       </c>
-      <c r="C12" s="98"/>
-      <c r="D12" s="98"/>
+      <c r="C12" s="108"/>
+      <c r="D12" s="108"/>
       <c r="E12" s="8">
         <v>1</v>
       </c>
@@ -4468,11 +4485,11 @@
       <c r="A13" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="B13" s="98" t="s">
+      <c r="B13" s="108" t="s">
         <v>92</v>
       </c>
-      <c r="C13" s="98"/>
-      <c r="D13" s="98"/>
+      <c r="C13" s="108"/>
+      <c r="D13" s="108"/>
       <c r="E13" s="8">
         <v>10</v>
       </c>
@@ -4485,11 +4502,11 @@
       <c r="A14" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="B14" s="98" t="s">
+      <c r="B14" s="108" t="s">
         <v>178</v>
       </c>
-      <c r="C14" s="98"/>
-      <c r="D14" s="98"/>
+      <c r="C14" s="108"/>
+      <c r="D14" s="108"/>
       <c r="E14" s="8">
         <v>4</v>
       </c>
@@ -4502,11 +4519,11 @@
       <c r="A15" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="B15" s="98" t="s">
+      <c r="B15" s="108" t="s">
         <v>179</v>
       </c>
-      <c r="C15" s="98"/>
-      <c r="D15" s="98"/>
+      <c r="C15" s="108"/>
+      <c r="D15" s="108"/>
       <c r="E15" s="8">
         <v>4</v>
       </c>
@@ -4519,11 +4536,11 @@
       <c r="A16" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="B16" s="98" t="s">
+      <c r="B16" s="108" t="s">
         <v>99</v>
       </c>
-      <c r="C16" s="98"/>
-      <c r="D16" s="98"/>
+      <c r="C16" s="108"/>
+      <c r="D16" s="108"/>
       <c r="E16" s="15">
         <v>4</v>
       </c>
@@ -4536,11 +4553,11 @@
       <c r="A17" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="B17" s="98" t="s">
+      <c r="B17" s="108" t="s">
         <v>159</v>
       </c>
-      <c r="C17" s="98"/>
-      <c r="D17" s="98"/>
+      <c r="C17" s="108"/>
+      <c r="D17" s="108"/>
       <c r="E17" s="8">
         <v>1</v>
       </c>
@@ -4553,11 +4570,11 @@
       <c r="A18" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="B18" s="98" t="s">
+      <c r="B18" s="108" t="s">
         <v>100</v>
       </c>
-      <c r="C18" s="98"/>
-      <c r="D18" s="98"/>
+      <c r="C18" s="108"/>
+      <c r="D18" s="108"/>
       <c r="E18" s="8">
         <v>1</v>
       </c>
@@ -4570,11 +4587,11 @@
       <c r="A19" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="B19" s="98" t="s">
+      <c r="B19" s="108" t="s">
         <v>101</v>
       </c>
-      <c r="C19" s="98"/>
-      <c r="D19" s="98"/>
+      <c r="C19" s="108"/>
+      <c r="D19" s="108"/>
       <c r="E19" s="8">
         <v>1</v>
       </c>
@@ -4587,11 +4604,11 @@
       <c r="A20" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="B20" s="98" t="s">
+      <c r="B20" s="108" t="s">
         <v>180</v>
       </c>
-      <c r="C20" s="98"/>
-      <c r="D20" s="98"/>
+      <c r="C20" s="108"/>
+      <c r="D20" s="108"/>
       <c r="E20" s="8">
         <v>1</v>
       </c>
@@ -4604,11 +4621,11 @@
       <c r="A21" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="B21" s="98" t="s">
+      <c r="B21" s="108" t="s">
         <v>176</v>
       </c>
-      <c r="C21" s="98"/>
-      <c r="D21" s="98"/>
+      <c r="C21" s="108"/>
+      <c r="D21" s="108"/>
       <c r="E21" s="15">
         <v>1</v>
       </c>
@@ -4621,11 +4638,11 @@
       <c r="A22" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="B22" s="98" t="s">
+      <c r="B22" s="108" t="s">
         <v>181</v>
       </c>
-      <c r="C22" s="98"/>
-      <c r="D22" s="98"/>
+      <c r="C22" s="108"/>
+      <c r="D22" s="108"/>
       <c r="E22" s="8">
         <v>12</v>
       </c>
@@ -4638,11 +4655,11 @@
       <c r="A23" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="B23" s="98" t="s">
+      <c r="B23" s="108" t="s">
         <v>177</v>
       </c>
-      <c r="C23" s="98"/>
-      <c r="D23" s="98"/>
+      <c r="C23" s="108"/>
+      <c r="D23" s="108"/>
       <c r="E23" s="7">
         <v>12</v>
       </c>
@@ -4655,11 +4672,11 @@
       <c r="A24" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="B24" s="98" t="s">
+      <c r="B24" s="108" t="s">
         <v>153</v>
       </c>
-      <c r="C24" s="98"/>
-      <c r="D24" s="98"/>
+      <c r="C24" s="108"/>
+      <c r="D24" s="108"/>
       <c r="E24" s="8">
         <v>20</v>
       </c>
@@ -4672,11 +4689,11 @@
       <c r="A25" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="B25" s="98" t="s">
+      <c r="B25" s="108" t="s">
         <v>154</v>
       </c>
-      <c r="C25" s="98"/>
-      <c r="D25" s="98"/>
+      <c r="C25" s="108"/>
+      <c r="D25" s="108"/>
       <c r="E25" s="8">
         <v>20</v>
       </c>
@@ -4689,11 +4706,11 @@
       <c r="A26" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="B26" s="98" t="s">
+      <c r="B26" s="108" t="s">
         <v>93</v>
       </c>
-      <c r="C26" s="98"/>
-      <c r="D26" s="98"/>
+      <c r="C26" s="108"/>
+      <c r="D26" s="108"/>
       <c r="E26" s="8">
         <v>12</v>
       </c>
@@ -4706,11 +4723,11 @@
       <c r="A27" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="B27" s="98" t="s">
+      <c r="B27" s="108" t="s">
         <v>147</v>
       </c>
-      <c r="C27" s="98"/>
-      <c r="D27" s="98"/>
+      <c r="C27" s="108"/>
+      <c r="D27" s="108"/>
       <c r="E27" s="8">
         <v>12</v>
       </c>
@@ -4723,11 +4740,11 @@
       <c r="A28" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="B28" s="98" t="s">
+      <c r="B28" s="108" t="s">
         <v>94</v>
       </c>
-      <c r="C28" s="98"/>
-      <c r="D28" s="98"/>
+      <c r="C28" s="108"/>
+      <c r="D28" s="108"/>
       <c r="E28" s="8">
         <v>20</v>
       </c>
@@ -4740,11 +4757,11 @@
       <c r="A29" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="B29" s="98" t="s">
+      <c r="B29" s="108" t="s">
         <v>95</v>
       </c>
-      <c r="C29" s="98"/>
-      <c r="D29" s="98"/>
+      <c r="C29" s="108"/>
+      <c r="D29" s="108"/>
       <c r="E29" s="8">
         <v>20</v>
       </c>
@@ -4757,11 +4774,11 @@
       <c r="A30" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="B30" s="98" t="s">
+      <c r="B30" s="108" t="s">
         <v>155</v>
       </c>
-      <c r="C30" s="98"/>
-      <c r="D30" s="98"/>
+      <c r="C30" s="108"/>
+      <c r="D30" s="108"/>
       <c r="E30" s="8">
         <v>20</v>
       </c>
@@ -4774,11 +4791,11 @@
       <c r="A31" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="B31" s="98" t="s">
+      <c r="B31" s="108" t="s">
         <v>96</v>
       </c>
-      <c r="C31" s="98"/>
-      <c r="D31" s="98"/>
+      <c r="C31" s="108"/>
+      <c r="D31" s="108"/>
       <c r="E31" s="8">
         <v>12</v>
       </c>
@@ -4791,11 +4808,11 @@
       <c r="A32" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="B32" s="98" t="s">
+      <c r="B32" s="108" t="s">
         <v>206</v>
       </c>
-      <c r="C32" s="98"/>
-      <c r="D32" s="98"/>
+      <c r="C32" s="108"/>
+      <c r="D32" s="108"/>
       <c r="E32" s="15">
         <v>1</v>
       </c>
@@ -4808,11 +4825,11 @@
       <c r="A33" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="B33" s="98" t="s">
+      <c r="B33" s="108" t="s">
         <v>156</v>
       </c>
-      <c r="C33" s="98"/>
-      <c r="D33" s="98"/>
+      <c r="C33" s="108"/>
+      <c r="D33" s="108"/>
       <c r="E33" s="15">
         <v>1</v>
       </c>
@@ -4825,11 +4842,11 @@
       <c r="A34" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="B34" s="98" t="s">
+      <c r="B34" s="108" t="s">
         <v>97</v>
       </c>
-      <c r="C34" s="98"/>
-      <c r="D34" s="98"/>
+      <c r="C34" s="108"/>
+      <c r="D34" s="108"/>
       <c r="E34" s="15">
         <v>1</v>
       </c>
@@ -4842,11 +4859,11 @@
       <c r="A35" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="B35" s="98" t="s">
+      <c r="B35" s="108" t="s">
         <v>98</v>
       </c>
-      <c r="C35" s="98"/>
-      <c r="D35" s="98"/>
+      <c r="C35" s="108"/>
+      <c r="D35" s="108"/>
       <c r="E35" s="15">
         <v>1</v>
       </c>
@@ -4859,11 +4876,11 @@
       <c r="A36" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="B36" s="98" t="s">
+      <c r="B36" s="108" t="s">
         <v>110</v>
       </c>
-      <c r="C36" s="98"/>
-      <c r="D36" s="98"/>
+      <c r="C36" s="108"/>
+      <c r="D36" s="108"/>
       <c r="E36" s="15">
         <v>1</v>
       </c>
@@ -4876,11 +4893,11 @@
       <c r="A37" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="B37" s="98" t="s">
+      <c r="B37" s="108" t="s">
         <v>108</v>
       </c>
-      <c r="C37" s="98"/>
-      <c r="D37" s="98"/>
+      <c r="C37" s="108"/>
+      <c r="D37" s="108"/>
       <c r="E37" s="15">
         <v>1</v>
       </c>
@@ -4893,11 +4910,11 @@
       <c r="A38" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="B38" s="98" t="s">
+      <c r="B38" s="108" t="s">
         <v>102</v>
       </c>
-      <c r="C38" s="98"/>
-      <c r="D38" s="98"/>
+      <c r="C38" s="108"/>
+      <c r="D38" s="108"/>
       <c r="E38" s="8">
         <v>20</v>
       </c>
@@ -4910,11 +4927,11 @@
       <c r="A39" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="B39" s="98" t="s">
+      <c r="B39" s="108" t="s">
         <v>103</v>
       </c>
-      <c r="C39" s="98"/>
-      <c r="D39" s="98"/>
+      <c r="C39" s="108"/>
+      <c r="D39" s="108"/>
       <c r="E39" s="15">
         <v>20</v>
       </c>
@@ -4927,11 +4944,11 @@
       <c r="A40" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="B40" s="98" t="s">
+      <c r="B40" s="108" t="s">
         <v>104</v>
       </c>
-      <c r="C40" s="98"/>
-      <c r="D40" s="98"/>
+      <c r="C40" s="108"/>
+      <c r="D40" s="108"/>
       <c r="E40" s="15">
         <v>20</v>
       </c>
@@ -4944,11 +4961,11 @@
       <c r="A41" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="B41" s="98" t="s">
+      <c r="B41" s="108" t="s">
         <v>105</v>
       </c>
-      <c r="C41" s="98"/>
-      <c r="D41" s="98"/>
+      <c r="C41" s="108"/>
+      <c r="D41" s="108"/>
       <c r="E41" s="15">
         <v>20</v>
       </c>
@@ -4961,11 +4978,11 @@
       <c r="A42" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="B42" s="98" t="s">
+      <c r="B42" s="108" t="s">
         <v>106</v>
       </c>
-      <c r="C42" s="98"/>
-      <c r="D42" s="98"/>
+      <c r="C42" s="108"/>
+      <c r="D42" s="108"/>
       <c r="E42" s="15">
         <v>1</v>
       </c>
@@ -4978,11 +4995,11 @@
       <c r="A43" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="B43" s="98" t="s">
+      <c r="B43" s="108" t="s">
         <v>107</v>
       </c>
-      <c r="C43" s="98"/>
-      <c r="D43" s="98"/>
+      <c r="C43" s="108"/>
+      <c r="D43" s="108"/>
       <c r="E43" s="15">
         <v>1</v>
       </c>
@@ -4995,11 +5012,11 @@
       <c r="A44" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="B44" s="98" t="s">
+      <c r="B44" s="108" t="s">
         <v>109</v>
       </c>
-      <c r="C44" s="98"/>
-      <c r="D44" s="98"/>
+      <c r="C44" s="108"/>
+      <c r="D44" s="108"/>
       <c r="E44" s="7">
         <v>1</v>
       </c>
@@ -5012,11 +5029,11 @@
       <c r="A45" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="B45" s="98" t="s">
+      <c r="B45" s="108" t="s">
         <v>160</v>
       </c>
-      <c r="C45" s="98"/>
-      <c r="D45" s="98"/>
+      <c r="C45" s="108"/>
+      <c r="D45" s="108"/>
       <c r="E45" s="7">
         <v>1</v>
       </c>
@@ -5029,9 +5046,9 @@
       <c r="A46" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="B46" s="104"/>
-      <c r="C46" s="104"/>
-      <c r="D46" s="104"/>
+      <c r="B46" s="109"/>
+      <c r="C46" s="109"/>
+      <c r="D46" s="109"/>
       <c r="E46" s="12"/>
       <c r="F46" s="16"/>
       <c r="G46" s="6"/>
@@ -5040,9 +5057,9 @@
       <c r="A47" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="B47" s="104"/>
-      <c r="C47" s="104"/>
-      <c r="D47" s="104"/>
+      <c r="B47" s="109"/>
+      <c r="C47" s="109"/>
+      <c r="D47" s="109"/>
       <c r="E47" s="12"/>
       <c r="F47" s="16"/>
       <c r="G47" s="6"/>
@@ -5051,9 +5068,9 @@
       <c r="A48" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="B48" s="103"/>
-      <c r="C48" s="103"/>
-      <c r="D48" s="103"/>
+      <c r="B48" s="110"/>
+      <c r="C48" s="110"/>
+      <c r="D48" s="110"/>
       <c r="E48" s="7"/>
       <c r="F48" s="7"/>
       <c r="G48" s="6"/>
@@ -5062,9 +5079,9 @@
       <c r="A49" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="B49" s="103"/>
-      <c r="C49" s="103"/>
-      <c r="D49" s="103"/>
+      <c r="B49" s="110"/>
+      <c r="C49" s="110"/>
+      <c r="D49" s="110"/>
       <c r="E49" s="7"/>
       <c r="F49" s="7"/>
       <c r="G49" s="6"/>
@@ -5073,9 +5090,9 @@
       <c r="A50" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="B50" s="103"/>
-      <c r="C50" s="103"/>
-      <c r="D50" s="103"/>
+      <c r="B50" s="110"/>
+      <c r="C50" s="110"/>
+      <c r="D50" s="110"/>
       <c r="E50" s="7"/>
       <c r="F50" s="7"/>
       <c r="G50" s="6"/>
@@ -5084,9 +5101,9 @@
       <c r="A51" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="B51" s="98"/>
-      <c r="C51" s="98"/>
-      <c r="D51" s="98"/>
+      <c r="B51" s="108"/>
+      <c r="C51" s="108"/>
+      <c r="D51" s="108"/>
       <c r="E51" s="7"/>
       <c r="F51" s="7"/>
       <c r="G51" s="6"/>
@@ -5095,9 +5112,9 @@
       <c r="A52" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="B52" s="98"/>
-      <c r="C52" s="98"/>
-      <c r="D52" s="98"/>
+      <c r="B52" s="108"/>
+      <c r="C52" s="108"/>
+      <c r="D52" s="108"/>
       <c r="E52" s="7"/>
       <c r="F52" s="7"/>
       <c r="G52" s="6"/>
@@ -5153,20 +5170,29 @@
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="C1:G1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="B49:D49"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B23:D23"/>
@@ -5183,29 +5209,20 @@
     <mergeCell ref="B38:D38"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="B48:D48"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="C1:G1"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.11811023622047245" right="0.11811023622047245" top="0.15748031496062992" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>